<commit_message>
Inclusão do script de alteração de BP's
</commit_message>
<xml_diff>
--- a/Planilhas/Ordens internas.xlsx
+++ b/Planilhas/Ordens internas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\Planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1AAEE5-883C-42F2-B998-35C8D8C7D899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D80876-BD0E-44C1-92BB-2352BA212076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28635" yWindow="-135" windowWidth="29130" windowHeight="15810" xr2:uid="{02AC0C7C-EFAF-4F40-9A5D-1FFDAF83D387}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{02AC0C7C-EFAF-4F40-9A5D-1FFDAF83D387}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="80">
   <si>
     <t>ID</t>
   </si>
@@ -62,199 +62,223 @@
     <t>IMO</t>
   </si>
   <si>
-    <t>100500004275-0</t>
-  </si>
-  <si>
-    <t>100500004276-0</t>
-  </si>
-  <si>
-    <t>100500004277-0</t>
-  </si>
-  <si>
-    <t>100500004278-0</t>
-  </si>
-  <si>
-    <t>100500004279-0</t>
-  </si>
-  <si>
-    <t>100500004280-0</t>
-  </si>
-  <si>
-    <t>100500004281-0</t>
-  </si>
-  <si>
-    <t>100500004282-0</t>
-  </si>
-  <si>
-    <t>100500004283-0</t>
-  </si>
-  <si>
-    <t>100500004284-0</t>
-  </si>
-  <si>
-    <t>100500004285-0</t>
-  </si>
-  <si>
-    <t>100500004286-0</t>
-  </si>
-  <si>
-    <t>100500004287-0</t>
-  </si>
-  <si>
-    <t>100500004288-0</t>
-  </si>
-  <si>
-    <t>100500004289-0</t>
-  </si>
-  <si>
-    <t>100300003684-0</t>
-  </si>
-  <si>
-    <t>100500004290-0</t>
-  </si>
-  <si>
-    <t>100500004291-0</t>
-  </si>
-  <si>
-    <t>100500004292-0</t>
-  </si>
-  <si>
-    <t>100500004293-0</t>
-  </si>
-  <si>
-    <t>100500004294-0</t>
-  </si>
-  <si>
-    <t>100500004295-0</t>
-  </si>
-  <si>
-    <t>100500004296-0</t>
-  </si>
-  <si>
-    <t>100500004297-0</t>
-  </si>
-  <si>
-    <t>100500004298-0</t>
-  </si>
-  <si>
-    <t>100500004299-0</t>
-  </si>
-  <si>
-    <t>100500004300-0</t>
-  </si>
-  <si>
-    <t>100500004301-0</t>
-  </si>
-  <si>
-    <t>100500004302-0</t>
-  </si>
-  <si>
-    <t>100500004303-0</t>
-  </si>
-  <si>
-    <t>100500004304-0</t>
-  </si>
-  <si>
-    <t>100500004305-0</t>
-  </si>
-  <si>
-    <t>100500004306-0</t>
-  </si>
-  <si>
-    <t>100500004307-0</t>
-  </si>
-  <si>
-    <t>100500004308-0</t>
-  </si>
-  <si>
-    <t>100500004309-0</t>
-  </si>
-  <si>
-    <t>100500004310-0</t>
-  </si>
-  <si>
-    <t>100500004311-0</t>
-  </si>
-  <si>
-    <t>100500004312-0</t>
-  </si>
-  <si>
-    <t>100500004313-0</t>
-  </si>
-  <si>
-    <t>100500004314-0</t>
-  </si>
-  <si>
-    <t>100500004315-0</t>
-  </si>
-  <si>
-    <t>100500004316-0</t>
-  </si>
-  <si>
-    <t>100500004317-0</t>
-  </si>
-  <si>
-    <t>100500004318-0</t>
-  </si>
-  <si>
-    <t>100500004319-0</t>
-  </si>
-  <si>
-    <t>100500004320-0</t>
-  </si>
-  <si>
-    <t>100500004321-0</t>
-  </si>
-  <si>
-    <t>100500004322-0</t>
-  </si>
-  <si>
-    <t>100500004323-0</t>
-  </si>
-  <si>
-    <t>100500004324-0</t>
-  </si>
-  <si>
-    <t>100500004325-0</t>
-  </si>
-  <si>
-    <t>100500004326-0</t>
-  </si>
-  <si>
-    <t>100500004327-0</t>
-  </si>
-  <si>
-    <t>100500004328-0</t>
-  </si>
-  <si>
-    <t>100500004329-0</t>
-  </si>
-  <si>
-    <t>100500004330-0</t>
-  </si>
-  <si>
-    <t>100500004331-0</t>
-  </si>
-  <si>
-    <t>100500004332-0</t>
-  </si>
-  <si>
-    <t>100500004333-0</t>
-  </si>
-  <si>
-    <t>100500004334-0</t>
-  </si>
-  <si>
-    <t>100500004335-0</t>
-  </si>
-  <si>
-    <t>100500004336-0</t>
-  </si>
-  <si>
-    <t>100500004337-0</t>
-  </si>
-  <si>
-    <t>100400000441-0</t>
+    <t>100300003704-0</t>
+  </si>
+  <si>
+    <t>100300003705-0</t>
+  </si>
+  <si>
+    <t>100300003706-0</t>
+  </si>
+  <si>
+    <t>100300003707-0</t>
+  </si>
+  <si>
+    <t>100300003708-0</t>
+  </si>
+  <si>
+    <t>100300003709-0</t>
+  </si>
+  <si>
+    <t>100300003710-0</t>
+  </si>
+  <si>
+    <t>100300003711-0</t>
+  </si>
+  <si>
+    <t>100300003712-0</t>
+  </si>
+  <si>
+    <t>100300003712-1</t>
+  </si>
+  <si>
+    <t>100300003713-0</t>
+  </si>
+  <si>
+    <t>100300003713-1</t>
+  </si>
+  <si>
+    <t>100300003714-0</t>
+  </si>
+  <si>
+    <t>100300003714-1</t>
+  </si>
+  <si>
+    <t>100300003715-0</t>
+  </si>
+  <si>
+    <t>100300003715-1</t>
+  </si>
+  <si>
+    <t>100300003716-0</t>
+  </si>
+  <si>
+    <t>100300003716-1</t>
+  </si>
+  <si>
+    <t>100300003717-0</t>
+  </si>
+  <si>
+    <t>100300003717-1</t>
+  </si>
+  <si>
+    <t>100300003718-0</t>
+  </si>
+  <si>
+    <t>100300003719-0</t>
+  </si>
+  <si>
+    <t>100300003720-0</t>
+  </si>
+  <si>
+    <t>100300003721-0</t>
+  </si>
+  <si>
+    <t>100300003722-0</t>
+  </si>
+  <si>
+    <t>100300003723-0</t>
+  </si>
+  <si>
+    <t>100300003720-1</t>
+  </si>
+  <si>
+    <t>100300003721-1</t>
+  </si>
+  <si>
+    <t>100300003722-1</t>
+  </si>
+  <si>
+    <t>100300003723-1</t>
+  </si>
+  <si>
+    <t>100300003724-0</t>
+  </si>
+  <si>
+    <t>100300003725-0</t>
+  </si>
+  <si>
+    <t>100300003726-0</t>
+  </si>
+  <si>
+    <t>100300003727-0</t>
+  </si>
+  <si>
+    <t>100300003728-0</t>
+  </si>
+  <si>
+    <t>100300003728-1</t>
+  </si>
+  <si>
+    <t>100300003728-2</t>
+  </si>
+  <si>
+    <t>100300003728-3</t>
+  </si>
+  <si>
+    <t>100300003729-0</t>
+  </si>
+  <si>
+    <t>100300003729-1</t>
+  </si>
+  <si>
+    <t>100300003729-2</t>
+  </si>
+  <si>
+    <t>100300003729-3</t>
+  </si>
+  <si>
+    <t>100300003730-0</t>
+  </si>
+  <si>
+    <t>100300003730-1</t>
+  </si>
+  <si>
+    <t>100300003730-2</t>
+  </si>
+  <si>
+    <t>100300003730-3</t>
+  </si>
+  <si>
+    <t>100300003731-0</t>
+  </si>
+  <si>
+    <t>100300003731-1</t>
+  </si>
+  <si>
+    <t>100300003731-2</t>
+  </si>
+  <si>
+    <t>100300003731-3</t>
+  </si>
+  <si>
+    <t>100300003732-0</t>
+  </si>
+  <si>
+    <t>100300003733-0</t>
+  </si>
+  <si>
+    <t>100300003734-0</t>
+  </si>
+  <si>
+    <t>100300003735-0</t>
+  </si>
+  <si>
+    <t>100300003732-1</t>
+  </si>
+  <si>
+    <t>100300003733-1</t>
+  </si>
+  <si>
+    <t>100300003734-1</t>
+  </si>
+  <si>
+    <t>100300003735-1</t>
+  </si>
+  <si>
+    <t>100300003732-2</t>
+  </si>
+  <si>
+    <t>100300003733-2</t>
+  </si>
+  <si>
+    <t>100300003734-2</t>
+  </si>
+  <si>
+    <t>100300003735-2</t>
+  </si>
+  <si>
+    <t>100300003736-0</t>
+  </si>
+  <si>
+    <t>100300003737-0</t>
+  </si>
+  <si>
+    <t>100300003738-0</t>
+  </si>
+  <si>
+    <t>100300003739-0</t>
+  </si>
+  <si>
+    <t>100300003736-1</t>
+  </si>
+  <si>
+    <t>100300003737-1</t>
+  </si>
+  <si>
+    <t>100300003738-1</t>
+  </si>
+  <si>
+    <t>100300003739-1</t>
+  </si>
+  <si>
+    <t>100300003740-0</t>
+  </si>
+  <si>
+    <t>100200000158-0</t>
+  </si>
+  <si>
+    <t>100400000443-0</t>
   </si>
 </sst>
 </file>
@@ -303,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -311,6 +335,9 @@
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,8 +465,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B4F3E30-B528-40FF-9409-54888BDB85B1}" name="Tabela1" displayName="Tabela1" ref="A1:F66" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="A1:F66" xr:uid="{2B4F3E30-B528-40FF-9409-54888BDB85B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B4F3E30-B528-40FF-9409-54888BDB85B1}" name="Tabela1" displayName="Tabela1" ref="A1:F74" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:F74" xr:uid="{2B4F3E30-B528-40FF-9409-54888BDB85B1}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C75EB0DB-1873-42F0-8DA5-476B8F47CD4C}" name="ORDEM" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{9E5B318B-80B2-4E12-B000-D16470013D94}" name="ID" dataDxfId="2"/>
@@ -769,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4A2C791-4A54-47ED-9039-9A1BBC31D39B}">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -802,7 +829,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B2" s="1">
         <v>2</v>
@@ -810,19 +837,19 @@
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2">
-        <v>120852</v>
+      <c r="F2" s="1">
+        <v>5665329</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B3" s="1">
         <v>3</v>
@@ -830,19 +857,19 @@
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
-      <c r="F3">
-        <v>181351</v>
+      <c r="F3" s="1">
+        <v>5665329</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B4" s="1">
         <v>4</v>
@@ -850,19 +877,19 @@
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4">
-        <v>96852</v>
+      <c r="F4" s="1">
+        <v>5665330</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B5" s="1">
         <v>5</v>
@@ -870,19 +897,19 @@
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5">
-        <v>96852</v>
+      <c r="F5" s="1">
+        <v>7587780</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B6" s="1">
         <v>6</v>
@@ -890,19 +917,19 @@
       <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
-        <v>96852</v>
+      <c r="F6" s="1">
+        <v>1147065</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B7" s="1">
         <v>7</v>
@@ -910,19 +937,19 @@
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="5" t="s">
         <v>12</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7">
-        <v>96852</v>
+      <c r="F7" s="1">
+        <v>1147065</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B8" s="1">
         <v>8</v>
@@ -930,19 +957,19 @@
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8">
-        <v>96852</v>
+      <c r="F8" s="1">
+        <v>1683371</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B9" s="1">
         <v>9</v>
@@ -950,19 +977,19 @@
       <c r="C9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9">
-        <v>96852</v>
+      <c r="F9" s="1">
+        <v>1683371</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B10" s="1">
         <v>10</v>
@@ -970,19 +997,19 @@
       <c r="C10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
-      <c r="F10">
-        <v>96852</v>
+      <c r="F10" s="1">
+        <v>376000</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B11" s="1">
         <v>11</v>
@@ -990,19 +1017,19 @@
       <c r="C11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>16</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
-      <c r="F11">
-        <v>96852</v>
+      <c r="F11" s="1">
+        <v>39750</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B12" s="1">
         <v>12</v>
@@ -1010,19 +1037,19 @@
       <c r="C12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
-      <c r="F12">
-        <v>96852</v>
+      <c r="F12" s="1">
+        <v>376000</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B13" s="1">
         <v>13</v>
@@ -1030,19 +1057,19 @@
       <c r="C13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
-      <c r="F13">
-        <v>96853</v>
+      <c r="F13" s="1">
+        <v>39750</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B14" s="1">
         <v>14</v>
@@ -1050,19 +1077,19 @@
       <c r="C14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
-      <c r="F14">
-        <v>96853</v>
+      <c r="F14" s="1">
+        <v>376000</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B15" s="1">
         <v>15</v>
@@ -1070,19 +1097,19 @@
       <c r="C15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
-      <c r="F15">
-        <v>96853</v>
+      <c r="F15" s="1">
+        <v>39750</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B16" s="1">
         <v>16</v>
@@ -1090,19 +1117,19 @@
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E16">
         <v>0</v>
       </c>
-      <c r="F16">
-        <v>96853</v>
+      <c r="F16" s="1">
+        <v>376000</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B17" s="1">
         <v>17</v>
@@ -1110,19 +1137,19 @@
       <c r="C17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E17">
         <v>0</v>
       </c>
-      <c r="F17">
-        <v>871917</v>
+      <c r="F17" s="1">
+        <v>39750</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B18" s="1">
         <v>18</v>
@@ -1130,19 +1157,19 @@
       <c r="C18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
-      <c r="F18">
-        <v>153366</v>
+      <c r="F18" s="1">
+        <v>628486</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B19" s="1">
         <v>19</v>
@@ -1150,19 +1177,19 @@
       <c r="C19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
-      <c r="F19">
-        <v>462713</v>
+      <c r="F19" s="1">
+        <v>14697</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B20" s="1">
         <v>20</v>
@@ -1170,19 +1197,19 @@
       <c r="C20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E20">
         <v>0</v>
       </c>
-      <c r="F20">
-        <v>187405</v>
+      <c r="F20" s="1">
+        <v>628486</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B21" s="1">
         <v>21</v>
@@ -1190,19 +1217,19 @@
       <c r="C21" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="5" t="s">
         <v>26</v>
       </c>
       <c r="E21">
         <v>0</v>
       </c>
-      <c r="F21">
-        <v>100391</v>
+      <c r="F21" s="1">
+        <v>14697</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B22" s="1">
         <v>22</v>
@@ -1210,19 +1237,19 @@
       <c r="C22" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="5" t="s">
         <v>27</v>
       </c>
       <c r="E22">
         <v>0</v>
       </c>
-      <c r="F22">
-        <v>100391</v>
+      <c r="F22" s="1">
+        <v>2022379</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B23" s="1">
         <v>23</v>
@@ -1230,19 +1257,19 @@
       <c r="C23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="5" t="s">
         <v>28</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
-      <c r="F23">
-        <v>100391</v>
+      <c r="F23" s="1">
+        <v>2022379</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B24" s="1">
         <v>24</v>
@@ -1250,19 +1277,19 @@
       <c r="C24" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="5" t="s">
         <v>29</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
-      <c r="F24">
-        <v>100391</v>
+      <c r="F24" s="1">
+        <v>6839726</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B25" s="1">
         <v>25</v>
@@ -1270,19 +1297,19 @@
       <c r="C25" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="5" t="s">
         <v>30</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
-      <c r="F25">
-        <v>80244</v>
+      <c r="F25" s="1">
+        <v>6839726</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B26" s="1">
         <v>26</v>
@@ -1290,19 +1317,19 @@
       <c r="C26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="5" t="s">
         <v>31</v>
       </c>
       <c r="E26">
         <v>0</v>
       </c>
-      <c r="F26">
-        <v>80245</v>
+      <c r="F26" s="1">
+        <v>6839725</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B27" s="1">
         <v>27</v>
@@ -1310,19 +1337,19 @@
       <c r="C27" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="5" t="s">
         <v>32</v>
       </c>
       <c r="E27">
         <v>0</v>
       </c>
-      <c r="F27">
-        <v>80245</v>
+      <c r="F27" s="1">
+        <v>6839725</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B28" s="1">
         <v>28</v>
@@ -1330,19 +1357,19 @@
       <c r="C28" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="5" t="s">
         <v>33</v>
       </c>
       <c r="E28">
         <v>0</v>
       </c>
-      <c r="F28">
-        <v>80245</v>
+      <c r="F28" s="1">
+        <v>544992</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B29" s="1">
         <v>29</v>
@@ -1350,19 +1377,19 @@
       <c r="C29" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E29">
         <v>0</v>
       </c>
-      <c r="F29">
-        <v>80245</v>
+      <c r="F29" s="1">
+        <v>544992</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B30" s="1">
         <v>30</v>
@@ -1370,19 +1397,19 @@
       <c r="C30" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="5" t="s">
         <v>35</v>
       </c>
       <c r="E30">
         <v>0</v>
       </c>
-      <c r="F30">
-        <v>80245</v>
+      <c r="F30" s="1">
+        <v>544992</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B31" s="1">
         <v>31</v>
@@ -1390,19 +1417,19 @@
       <c r="C31" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="5" t="s">
         <v>36</v>
       </c>
       <c r="E31">
         <v>0</v>
       </c>
-      <c r="F31">
-        <v>80245</v>
+      <c r="F31" s="1">
+        <v>544992</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B32" s="1">
         <v>32</v>
@@ -1410,19 +1437,19 @@
       <c r="C32" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="5" t="s">
         <v>37</v>
       </c>
       <c r="E32">
         <v>0</v>
       </c>
-      <c r="F32">
-        <v>80245</v>
+      <c r="F32" s="1">
+        <v>17104733</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B33" s="1">
         <v>33</v>
@@ -1430,19 +1457,19 @@
       <c r="C33" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E33">
         <v>0</v>
       </c>
-      <c r="F33">
-        <v>66900</v>
+      <c r="F33" s="1">
+        <v>10221281</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B34" s="1">
         <v>34</v>
@@ -1450,19 +1477,19 @@
       <c r="C34" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="5" t="s">
         <v>39</v>
       </c>
       <c r="E34">
         <v>0</v>
       </c>
-      <c r="F34">
-        <v>66900</v>
+      <c r="F34" s="1">
+        <v>10221281</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B35" s="1">
         <v>35</v>
@@ -1470,19 +1497,19 @@
       <c r="C35" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="5" t="s">
         <v>40</v>
       </c>
       <c r="E35">
         <v>0</v>
       </c>
-      <c r="F35">
-        <v>125800</v>
+      <c r="F35" s="1">
+        <v>10221280</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B36" s="1">
         <v>36</v>
@@ -1490,19 +1517,19 @@
       <c r="C36" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="5" t="s">
         <v>41</v>
       </c>
       <c r="E36">
         <v>0</v>
       </c>
-      <c r="F36">
-        <v>125800</v>
+      <c r="F36" s="1">
+        <v>32072884</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B37" s="1">
         <v>37</v>
@@ -1510,19 +1537,19 @@
       <c r="C37" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="5" t="s">
         <v>42</v>
       </c>
       <c r="E37">
         <v>0</v>
       </c>
-      <c r="F37">
-        <v>125800</v>
+      <c r="F37" s="1">
+        <v>3227604</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B38" s="1">
         <v>38</v>
@@ -1530,19 +1557,19 @@
       <c r="C38" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="5" t="s">
         <v>43</v>
       </c>
       <c r="E38">
         <v>0</v>
       </c>
-      <c r="F38">
-        <v>125800</v>
+      <c r="F38" s="1">
+        <v>1781827</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B39" s="1">
         <v>39</v>
@@ -1550,19 +1577,19 @@
       <c r="C39" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="5" t="s">
         <v>44</v>
       </c>
       <c r="E39">
         <v>0</v>
       </c>
-      <c r="F39">
-        <v>125800</v>
+      <c r="F39" s="1">
+        <v>754650</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B40" s="1">
         <v>40</v>
@@ -1570,19 +1597,19 @@
       <c r="C40" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E40">
         <v>0</v>
       </c>
-      <c r="F40">
-        <v>125800</v>
+      <c r="F40" s="1">
+        <v>18091533</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B41" s="1">
         <v>41</v>
@@ -1590,19 +1617,19 @@
       <c r="C41" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="5" t="s">
         <v>46</v>
       </c>
       <c r="E41">
         <v>0</v>
       </c>
-      <c r="F41">
-        <v>125800</v>
+      <c r="F41" s="1">
+        <v>3227604</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B42" s="1">
         <v>42</v>
@@ -1610,19 +1637,19 @@
       <c r="C42" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="5" t="s">
         <v>47</v>
       </c>
       <c r="E42">
         <v>0</v>
       </c>
-      <c r="F42">
-        <v>125800</v>
+      <c r="F42" s="1">
+        <v>1781827</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B43" s="1">
         <v>43</v>
@@ -1630,19 +1657,19 @@
       <c r="C43" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="5" t="s">
         <v>48</v>
       </c>
       <c r="E43">
         <v>0</v>
       </c>
-      <c r="F43">
-        <v>125800</v>
+      <c r="F43" s="1">
+        <v>377325</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B44" s="1">
         <v>44</v>
@@ -1650,19 +1677,19 @@
       <c r="C44" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="5" t="s">
         <v>49</v>
       </c>
       <c r="E44">
         <v>0</v>
       </c>
-      <c r="F44">
-        <v>125800</v>
+      <c r="F44" s="1">
+        <v>35636537</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B45" s="1">
         <v>45</v>
@@ -1670,19 +1697,19 @@
       <c r="C45" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="5" t="s">
         <v>50</v>
       </c>
       <c r="E45">
         <v>0</v>
       </c>
-      <c r="F45">
-        <v>125800</v>
+      <c r="F45" s="1">
+        <v>3227605</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B46" s="1">
         <v>46</v>
@@ -1690,19 +1717,19 @@
       <c r="C46" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="5" t="s">
         <v>51</v>
       </c>
       <c r="E46">
         <v>0</v>
       </c>
-      <c r="F46">
-        <v>125800</v>
+      <c r="F46" s="1">
+        <v>1781827</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B47" s="1">
         <v>47</v>
@@ -1710,19 +1737,19 @@
       <c r="C47" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="5" t="s">
         <v>52</v>
       </c>
       <c r="E47">
         <v>0</v>
       </c>
-      <c r="F47">
-        <v>125800</v>
+      <c r="F47" s="1">
+        <v>377325</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B48" s="1">
         <v>48</v>
@@ -1730,19 +1757,19 @@
       <c r="C48" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" s="5" t="s">
         <v>53</v>
       </c>
       <c r="E48">
         <v>0</v>
       </c>
-      <c r="F48">
-        <v>125800</v>
+      <c r="F48" s="1">
+        <v>35636538</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B49" s="1">
         <v>49</v>
@@ -1750,19 +1777,19 @@
       <c r="C49" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" s="5" t="s">
         <v>54</v>
       </c>
       <c r="E49">
         <v>0</v>
       </c>
-      <c r="F49">
-        <v>106200</v>
+      <c r="F49" s="1">
+        <v>3227605</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B50" s="1">
         <v>50</v>
@@ -1770,19 +1797,19 @@
       <c r="C50" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="5" t="s">
         <v>55</v>
       </c>
       <c r="E50">
         <v>0</v>
       </c>
-      <c r="F50">
-        <v>117700</v>
+      <c r="F50" s="1">
+        <v>1781827</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B51" s="1">
         <v>51</v>
@@ -1790,19 +1817,19 @@
       <c r="C51" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="5" t="s">
         <v>56</v>
       </c>
       <c r="E51">
         <v>0</v>
       </c>
-      <c r="F51">
-        <v>70066</v>
+      <c r="F51" s="1">
+        <v>580500</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B52" s="1">
         <v>52</v>
@@ -1810,19 +1837,19 @@
       <c r="C52" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D52" s="5" t="s">
         <v>57</v>
       </c>
       <c r="E52">
         <v>0</v>
       </c>
-      <c r="F52">
-        <v>70066</v>
+      <c r="F52" s="1">
+        <v>2486556</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B53" s="1">
         <v>53</v>
@@ -1830,19 +1857,19 @@
       <c r="C53" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D53" s="5" t="s">
         <v>58</v>
       </c>
       <c r="E53">
         <v>0</v>
       </c>
-      <c r="F53">
-        <v>70066</v>
+      <c r="F53" s="1">
+        <v>2486556</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B54" s="1">
         <v>54</v>
@@ -1850,19 +1877,19 @@
       <c r="C54" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D54" s="5" t="s">
         <v>59</v>
       </c>
       <c r="E54">
         <v>0</v>
       </c>
-      <c r="F54">
-        <v>70066</v>
+      <c r="F54" s="1">
+        <v>2486557</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B55" s="1">
         <v>55</v>
@@ -1870,19 +1897,19 @@
       <c r="C55" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D55" s="5" t="s">
         <v>60</v>
       </c>
       <c r="E55">
         <v>0</v>
       </c>
-      <c r="F55">
-        <v>70067</v>
+      <c r="F55" s="1">
+        <v>2486557</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B56" s="1">
         <v>56</v>
@@ -1890,19 +1917,19 @@
       <c r="C56" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D56" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E56">
         <v>0</v>
       </c>
-      <c r="F56">
-        <v>70067</v>
+      <c r="F56" s="1">
+        <v>1722623</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B57" s="1">
         <v>57</v>
@@ -1910,19 +1937,19 @@
       <c r="C57" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D57" s="5" t="s">
         <v>62</v>
       </c>
       <c r="E57">
         <v>0</v>
       </c>
-      <c r="F57">
-        <v>70067</v>
+      <c r="F57" s="1">
+        <v>1722623</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B58" s="1">
         <v>58</v>
@@ -1930,19 +1957,19 @@
       <c r="C58" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D58" s="5" t="s">
         <v>63</v>
       </c>
       <c r="E58">
         <v>0</v>
       </c>
-      <c r="F58">
-        <v>70067</v>
+      <c r="F58" s="1">
+        <v>1722623</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B59" s="1">
         <v>59</v>
@@ -1950,19 +1977,19 @@
       <c r="C59" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D59" s="5" t="s">
         <v>64</v>
       </c>
       <c r="E59">
         <v>0</v>
       </c>
-      <c r="F59">
-        <v>70067</v>
+      <c r="F59" s="1">
+        <v>1722623</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B60" s="1">
         <v>60</v>
@@ -1970,19 +1997,19 @@
       <c r="C60" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D60" s="5" t="s">
         <v>65</v>
       </c>
       <c r="E60">
         <v>0</v>
       </c>
-      <c r="F60">
-        <v>70067</v>
+      <c r="F60" s="1">
+        <v>1086718</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B61" s="1">
         <v>61</v>
@@ -1990,19 +2017,19 @@
       <c r="C61" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D61" s="5" t="s">
         <v>66</v>
       </c>
       <c r="E61">
         <v>0</v>
       </c>
-      <c r="F61">
-        <v>70067</v>
+      <c r="F61" s="1">
+        <v>1086718</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B62" s="1">
         <v>62</v>
@@ -2010,19 +2037,19 @@
       <c r="C62" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D62" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E62">
         <v>0</v>
       </c>
-      <c r="F62">
-        <v>70067</v>
+      <c r="F62" s="1">
+        <v>1086718</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B63" s="1">
         <v>63</v>
@@ -2030,19 +2057,19 @@
       <c r="C63" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D63" t="s">
+      <c r="D63" s="5" t="s">
         <v>68</v>
       </c>
       <c r="E63">
         <v>0</v>
       </c>
-      <c r="F63">
-        <v>114900</v>
+      <c r="F63" s="1">
+        <v>1086718</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B64" s="1">
         <v>64</v>
@@ -2050,19 +2077,19 @@
       <c r="C64" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D64" t="s">
+      <c r="D64" s="5" t="s">
         <v>69</v>
       </c>
       <c r="E64">
         <v>0</v>
       </c>
-      <c r="F64">
-        <v>55000</v>
+      <c r="F64" s="1">
+        <v>4165498</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B65" s="1">
         <v>65</v>
@@ -2070,19 +2097,19 @@
       <c r="C65" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D65" t="s">
+      <c r="D65" s="5" t="s">
         <v>70</v>
       </c>
       <c r="E65">
         <v>0</v>
       </c>
-      <c r="F65">
-        <v>55000</v>
+      <c r="F65" s="1">
+        <v>4165498</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66">
-        <v>600023</v>
+        <v>600032</v>
       </c>
       <c r="B66" s="1">
         <v>66</v>
@@ -2090,14 +2117,174 @@
       <c r="C66" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D66" t="s">
+      <c r="D66" s="5" t="s">
         <v>71</v>
       </c>
       <c r="E66">
         <v>0</v>
       </c>
-      <c r="F66">
-        <v>2516862.0000000005</v>
+      <c r="F66" s="1">
+        <v>4165499</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>600032</v>
+      </c>
+      <c r="B67" s="1">
+        <v>67</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67" s="1">
+        <v>4165499</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>600032</v>
+      </c>
+      <c r="B68" s="1">
+        <v>68</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68" s="1">
+        <v>3157878</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>600032</v>
+      </c>
+      <c r="B69" s="1">
+        <v>69</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69" s="1">
+        <v>3157879</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>600032</v>
+      </c>
+      <c r="B70" s="1">
+        <v>70</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70" s="1">
+        <v>3157879</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>600032</v>
+      </c>
+      <c r="B71" s="1">
+        <v>71</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+      <c r="F71" s="1">
+        <v>3157879</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>600032</v>
+      </c>
+      <c r="B72" s="1">
+        <v>72</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72" s="1">
+        <v>2414634</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>600032</v>
+      </c>
+      <c r="B73" s="1">
+        <v>73</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73" s="1">
+        <v>273082253</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>600032</v>
+      </c>
+      <c r="B74" s="1">
+        <v>74</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74" s="1">
+        <v>260803653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>